<commit_message>
LoRa execution with results
</commit_message>
<xml_diff>
--- a/log_resuts.xlsx
+++ b/log_resuts.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -555,6 +555,57 @@
         <v>0.8953185955786735</v>
       </c>
       <c r="O2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-07 22:57:41</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>distilbert-base-uncased</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>48</v>
+      </c>
+      <c r="D3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E3" t="n">
+        <v>32</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>q_lin,v_lin</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="I3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J3" t="n">
+        <v>8</v>
+      </c>
+      <c r="K3" t="n">
+        <v>3</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2244.61</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.3796542286872864</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.9040962288686606</v>
+      </c>
+      <c r="O3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>